<commit_message>
Tier-2 audit complete: Virtu confirmed with QR(Undergrad NY)+QT internships added to Excel; Trexquant/GSA/Teza/Wolverine/Vatic/Selini/Balyasny/Headlands findings documented in notes
</commit_message>
<xml_diff>
--- a/Tier1_US_QR_QT_Internships.xlsx
+++ b/Tier1_US_QR_QT_Internships.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -514,7 +514,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>US Summer 2027 QR / QT Internships - Tier-1 New Targets (Jing Xiang Xu) - compiled 2026-10-03</t>
+          <t>US Summer 2027 QR / QT Internships - Tier-1+2 New Targets (11 firms) (Jing Xiang Xu) - compiled 2026-10-03</t>
         </is>
       </c>
     </row>
@@ -920,48 +920,136 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Virtu Financial</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>2027 Internship - Quantitative Researcher (Undergrad), 10 weeks Jun 7-Aug 13</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Open now</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/virtu/jobs/8142539002</t>
+        </is>
+      </c>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>D:\zcode\hk-dashboard\cv\Xu_Jingxiang_Virtu_QR_CV.pdf</t>
+        </is>
+      </c>
+      <c r="H13" s="12" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Virtu Financial</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>2027 Internship - Quantitative Trading</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Austin / Chicago / New York</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Open now</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/virtu/jobs/8624408002?gh_jid=8624408002</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>D:\zcode\hk-dashboard\cv\Xu_Jingxiang_Virtu_QT_CV.pdf</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
         <is>
           <t>Notes:</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="14" t="inlineStr">
-        <is>
-          <t>1. All 9 postings verified live on 2026-10-03 via quantroles.com hidden-gems audit (cross-checked against the 56-firm applied list - none duplicated).</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="14" t="inlineStr">
-        <is>
-          <t>2. Deadlines are rolling - seats fill without notice (Deutsche Bank closed 3 weeks early). Apply in list order: QR-fit firms first (Voloridge, Anthelion, Stevens), then QT (TransMarket, BlackEdge, All Options, Group One, Kershner), then PEAK6 bootcamp.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>3. CVs are the in-place-tailored one-page PDFs in D:\zcode\hk-dashboard\cv\ (trading template for QT roles, quant-research template for QR roles).</t>
+          <t>1. All 9 postings verified live on 2026-10-03 via quantroles.com hidden-gems audit (cross-checked against the 56-firm applied list - none duplicated).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>
+          <t>2. Deadlines are rolling - seats fill without notice (Deutsche Bank closed 3 weeks early). Apply in list order: QR-fit firms first (Voloridge, Anthelion, Stevens), then QT (TransMarket, BlackEdge, All Options, Group One, Kershner), then PEAK6 bootcamp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>3. CVs are the in-place-tailored one-page PDFs in D:\zcode\hk-dashboard\cv\ (trading template for QT roles, quant-research template for QR roles).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
           <t>4. Jump / Tower / HRT excluded from this sheet - already self-applying (tracked in the main dashboard).</t>
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>5. Tier-2 audit results: Virtu CONFIRMED (rows 10-11). Trexquant QR intern on LinkedIn (actively hiring, no public apply link - search Trexquant on LinkedIn). Balyasny/Headlands: QR internships exist but 2027 cycle unconfirmed or PhD-only. GSA: QR intern is London-only (NY is full-time). Teza: no intern role on Ashby board (QR All Streams is full-time). Wolverine: no intern postings live on wolve.com. Vatic/Selini: no intern roles. Wintermute: grad algo trader London only. Old Mission: QT 2027 Graduate full-time only. PDT/Voleon/Radix/CTC/Pinely/Qube-US: no public intern postings (Qube has QR&amp;T intern in SINGAPORE).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A18:H18"/>
-    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="A20:H20"/>
     <mergeCell ref="A16:H16"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A19:H19"/>
     <mergeCell ref="A17:H17"/>
   </mergeCells>
   <hyperlinks>
@@ -974,6 +1062,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Excel: add 4 US QD internships (Old Mission, Quantbot NY, InfiniteQuant, Quantic) with CVs; total 16 postings across 13 firms
</commit_message>
<xml_diff>
--- a/Tier1_US_QR_QT_Internships.xlsx
+++ b/Tier1_US_QR_QT_Internships.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -514,7 +514,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>US Summer 2027 QR / QT Internships - Tier-1+2 New Targets (11 firms) (Jing Xiang Xu) - compiled 2026-10-03</t>
+          <t>US Summer 2027 QR / QT Internships - Tier-1+2 New Targets (15 firms incl. QD) (Jing Xiang Xu) - compiled 2026-10-03</t>
         </is>
       </c>
     </row>
@@ -1000,57 +1000,225 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Old Mission Capital</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Software Engineer - 2027 Internship Program (June Start, trading-firm SWE/QD)</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Chicago, IL</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Open now</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>https://www.oldmissioncapital.com/careers/?gh_jid=7796180003</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>D:\zcode\hk-dashboard\cv\Xu_Jingxiang_OldMission_CV.pdf</t>
+        </is>
+      </c>
+      <c r="H15" s="12" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Quantbot Technologies</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Quantitative Developer Internship - 2027</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Open now</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>https://www.quantbot.com/careers/4341038009?gh_jid=4341038009</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>D:\zcode\hk-dashboard\cv\Xu_Jingxiang_Quantbot_QD_CV.pdf</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>InfiniteQuant</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Quantitative Developer Internship - Summer 2027</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 deadline</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>https://jobright.ai</t>
+        </is>
+      </c>
+      <c r="G17" s="11" t="inlineStr">
+        <is>
+          <t>D:\zcode\hk-dashboard\cv\Xu_Jingxiang_InfiniteQuant_CV.pdf</t>
+        </is>
+      </c>
+      <c r="H17" s="12" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Quantic</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Quantitative Developer Intern - Summer 2027 (10 weeks)</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Boston, MA</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Open now</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>https://www.quantic.com</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>D:\zcode\hk-dashboard\cv\Xu_Jingxiang_Quantic_CV.pdf</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
         <is>
           <t>Notes:</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="14" t="inlineStr">
-        <is>
-          <t>1. All 9 postings verified live on 2026-10-03 via quantroles.com hidden-gems audit (cross-checked against the 56-firm applied list - none duplicated).</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="14" t="inlineStr">
-        <is>
-          <t>2. Deadlines are rolling - seats fill without notice (Deutsche Bank closed 3 weeks early). Apply in list order: QR-fit firms first (Voloridge, Anthelion, Stevens), then QT (TransMarket, BlackEdge, All Options, Group One, Kershner), then PEAK6 bootcamp.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="14" t="inlineStr">
-        <is>
-          <t>3. CVs are the in-place-tailored one-page PDFs in D:\zcode\hk-dashboard\cv\ (trading template for QT roles, quant-research template for QR roles).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="14" t="inlineStr">
-        <is>
-          <t>4. Jump / Tower / HRT excluded from this sheet - already self-applying (tracked in the main dashboard).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>5. Tier-2 audit results: Virtu CONFIRMED (rows 10-11). Trexquant QR intern on LinkedIn (actively hiring, no public apply link - search Trexquant on LinkedIn). Balyasny/Headlands: QR internships exist but 2027 cycle unconfirmed or PhD-only. GSA: QR intern is London-only (NY is full-time). Teza: no intern role on Ashby board (QR All Streams is full-time). Wolverine: no intern postings live on wolve.com. Vatic/Selini: no intern roles. Wintermute: grad algo trader London only. Old Mission: QT 2027 Graduate full-time only. PDT/Voleon/Radix/CTC/Pinely/Qube-US: no public intern postings (Qube has QR&amp;T intern in SINGAPORE).</t>
+          <t>1. All 9 postings verified live on 2026-10-03 via quantroles.com hidden-gems audit (cross-checked against the 56-firm applied list - none duplicated).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t>2. Deadlines are rolling - seats fill without notice (Deutsche Bank closed 3 weeks early). Apply in list order: QR-fit firms first (Voloridge, Anthelion, Stevens), then QT (TransMarket, BlackEdge, All Options, Group One, Kershner), then PEAK6 bootcamp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>3. CVs are the in-place-tailored one-page PDFs in D:\zcode\hk-dashboard\cv\ (trading template for QT roles, quant-research template for QR roles).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>4. Jump / Tower / HRT excluded from this sheet - already self-applying (tracked in the main dashboard).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>5. QD additions (user request): Old Mission / Quantbot / InfiniteQuant / Quantic added - US QD internships found beyond the 69+11 firms. Point72 QSD intern EXCLUDED - JD is systems programming (Linux kernel/compilers), not quant research infra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>7. Tier-2 audit results: Virtu CONFIRMED (rows 10-11). Trexquant QR intern on LinkedIn (actively hiring, no public apply link - search Trexquant on LinkedIn). Balyasny/Headlands: QR internships exist but 2027 cycle unconfirmed or PhD-only. GSA: QR intern is London-only (NY is full-time). Teza: no intern role on Ashby board. Wolverine: no intern postings live on wolve.com. Vatic/Selini: no intern roles. Wintermute: grad algo trader London only. Old Mission QT 2027 Graduate full-time also live. PDT/Voleon/Radix/CTC/Pinely/Qube-US: no public intern postings (Qube has QR&amp;T intern in SINGAPORE).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A18:H18"/>
+  <mergeCells count="8">
+    <mergeCell ref="A26:H26"/>
     <mergeCell ref="A21:H21"/>
+    <mergeCell ref="A25:H25"/>
     <mergeCell ref="A20:H20"/>
-    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A24:H24"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A19:H19"/>
-    <mergeCell ref="A17:H17"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="A22:H22"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId1"/>
@@ -1064,6 +1232,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>